<commit_message>
Atribuciones sin marcas de plantilla: se resuelven al generar el paquete de datos, la API, las cestas, la vista de citas y los catálogos; control en check-licenses
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WpevEvgxxTSUSU4BwGMDZh
</commit_message>
<xml_diff>
--- a/data/pack/ca/avena.xlsx
+++ b/data/pack/ca/avena.xlsx
@@ -545,7 +545,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2800,7 +2800,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3185,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3405,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3625,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3680,7 +3680,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3790,7 +3790,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3955,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4175,7 +4175,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4285,7 +4285,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4340,7 +4340,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4615,7 +4615,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4670,7 +4670,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4725,7 +4725,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4780,7 +4780,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5605,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5715,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5825,7 +5825,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5935,7 +5935,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6155,7 +6155,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6210,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6265,7 +6265,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6375,7 +6375,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6485,7 +6485,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6595,7 +6595,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6815,7 +6815,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6870,7 +6870,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6925,7 +6925,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7090,7 +7090,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7145,7 +7145,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7255,7 +7255,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7310,7 +7310,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7475,7 +7475,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7695,7 +7695,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7915,7 +7915,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8025,7 +8025,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8135,7 +8135,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8190,7 +8190,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8300,7 +8300,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8355,7 +8355,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8465,7 +8465,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8575,7 +8575,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8630,7 +8630,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8685,7 +8685,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8740,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8795,7 +8795,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8905,7 +8905,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9125,7 +9125,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9180,7 +9180,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9235,7 +9235,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9345,7 +9345,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9455,7 +9455,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9565,7 +9565,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9675,7 +9675,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9730,7 +9730,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9785,7 +9785,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9840,7 +9840,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9895,7 +9895,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -9950,7 +9950,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10005,7 +10005,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10115,7 +10115,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10170,7 +10170,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10225,7 +10225,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10280,7 +10280,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10335,7 +10335,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10390,7 +10390,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10445,7 +10445,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10500,7 +10500,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10555,7 +10555,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10610,7 +10610,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10665,7 +10665,7 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10720,7 +10720,7 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10775,7 +10775,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10830,7 +10830,7 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10885,7 +10885,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10940,7 +10940,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -10995,7 +10995,7 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11050,7 +11050,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11105,7 +11105,7 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11160,7 +11160,7 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11215,7 +11215,7 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11325,7 +11325,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11380,7 +11380,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11435,7 +11435,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11490,7 +11490,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11545,7 +11545,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11600,7 +11600,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11655,7 +11655,7 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11710,7 +11710,7 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11765,7 +11765,7 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11820,7 +11820,7 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11875,7 +11875,7 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11930,7 +11930,7 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -11985,7 +11985,7 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12040,7 +12040,7 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12095,7 +12095,7 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12150,7 +12150,7 @@
       </c>
       <c r="K213" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12205,7 +12205,7 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12260,7 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12315,7 +12315,7 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12370,7 +12370,7 @@
       </c>
       <c r="K217" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12425,7 +12425,7 @@
       </c>
       <c r="K218" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12480,7 +12480,7 @@
       </c>
       <c r="K219" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12535,7 +12535,7 @@
       </c>
       <c r="K220" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12590,7 +12590,7 @@
       </c>
       <c r="K221" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12645,7 +12645,7 @@
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12700,7 +12700,7 @@
       </c>
       <c r="K223" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12755,7 +12755,7 @@
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12810,7 +12810,7 @@
       </c>
       <c r="K225" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12865,7 +12865,7 @@
       </c>
       <c r="K226" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12920,7 +12920,7 @@
       </c>
       <c r="K227" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -12975,7 +12975,7 @@
       </c>
       <c r="K228" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13030,7 +13030,7 @@
       </c>
       <c r="K229" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13085,7 +13085,7 @@
       </c>
       <c r="K230" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13140,7 +13140,7 @@
       </c>
       <c r="K231" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13195,7 +13195,7 @@
       </c>
       <c r="K232" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13250,7 +13250,7 @@
       </c>
       <c r="K233" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13305,7 +13305,7 @@
       </c>
       <c r="K234" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13360,7 +13360,7 @@
       </c>
       <c r="K235" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13415,7 +13415,7 @@
       </c>
       <c r="K236" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13470,7 +13470,7 @@
       </c>
       <c r="K237" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13525,7 +13525,7 @@
       </c>
       <c r="K238" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13580,7 +13580,7 @@
       </c>
       <c r="K239" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13635,7 +13635,7 @@
       </c>
       <c r="K240" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13690,7 +13690,7 @@
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13745,7 +13745,7 @@
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13800,7 +13800,7 @@
       </c>
       <c r="K243" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13855,7 +13855,7 @@
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13910,7 +13910,7 @@
       </c>
       <c r="K245" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -13965,7 +13965,7 @@
       </c>
       <c r="K246" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14020,7 +14020,7 @@
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14075,7 +14075,7 @@
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14130,7 +14130,7 @@
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14185,7 +14185,7 @@
       </c>
       <c r="K250" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14240,7 +14240,7 @@
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14295,7 +14295,7 @@
       </c>
       <c r="K252" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14350,7 +14350,7 @@
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14405,7 +14405,7 @@
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14460,7 +14460,7 @@
       </c>
       <c r="K255" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14515,7 +14515,7 @@
       </c>
       <c r="K256" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14570,7 +14570,7 @@
       </c>
       <c r="K257" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14625,7 +14625,7 @@
       </c>
       <c r="K258" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14680,7 +14680,7 @@
       </c>
       <c r="K259" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14735,7 +14735,7 @@
       </c>
       <c r="K260" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14790,7 +14790,7 @@
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14845,7 +14845,7 @@
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14900,7 +14900,7 @@
       </c>
       <c r="K263" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -14955,7 +14955,7 @@
       </c>
       <c r="K264" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15010,7 +15010,7 @@
       </c>
       <c r="K265" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15065,7 +15065,7 @@
       </c>
       <c r="K266" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15120,7 +15120,7 @@
       </c>
       <c r="K267" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15175,7 +15175,7 @@
       </c>
       <c r="K268" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15230,7 +15230,7 @@
       </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15285,7 +15285,7 @@
       </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15340,7 +15340,7 @@
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15395,7 +15395,7 @@
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15450,7 +15450,7 @@
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15505,7 +15505,7 @@
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15560,7 +15560,7 @@
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15615,7 +15615,7 @@
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15670,7 +15670,7 @@
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15725,7 +15725,7 @@
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15780,7 +15780,7 @@
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15835,7 +15835,7 @@
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15890,7 +15890,7 @@
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -15945,7 +15945,7 @@
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16000,7 +16000,7 @@
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16055,7 +16055,7 @@
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16110,7 +16110,7 @@
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16165,7 +16165,7 @@
       </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16220,7 +16220,7 @@
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16275,7 +16275,7 @@
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16330,7 +16330,7 @@
       </c>
       <c r="K289" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16385,7 +16385,7 @@
       </c>
       <c r="K290" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16440,7 +16440,7 @@
       </c>
       <c r="K291" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16495,7 +16495,7 @@
       </c>
       <c r="K292" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16550,7 +16550,7 @@
       </c>
       <c r="K293" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16605,7 +16605,7 @@
       </c>
       <c r="K294" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16660,7 +16660,7 @@
       </c>
       <c r="K295" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16715,7 +16715,7 @@
       </c>
       <c r="K296" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16770,7 +16770,7 @@
       </c>
       <c r="K297" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16825,7 +16825,7 @@
       </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16935,7 +16935,7 @@
       </c>
       <c r="K300" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -16990,7 +16990,7 @@
       </c>
       <c r="K301" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17045,7 +17045,7 @@
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17100,7 +17100,7 @@
       </c>
       <c r="K303" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17155,7 +17155,7 @@
       </c>
       <c r="K304" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17210,7 +17210,7 @@
       </c>
       <c r="K305" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17265,7 +17265,7 @@
       </c>
       <c r="K306" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17320,7 +17320,7 @@
       </c>
       <c r="K307" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17375,7 +17375,7 @@
       </c>
       <c r="K308" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17430,7 +17430,7 @@
       </c>
       <c r="K309" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17485,7 +17485,7 @@
       </c>
       <c r="K310" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17540,7 +17540,7 @@
       </c>
       <c r="K311" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17595,7 +17595,7 @@
       </c>
       <c r="K312" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17650,7 +17650,7 @@
       </c>
       <c r="K313" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17705,7 +17705,7 @@
       </c>
       <c r="K314" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17760,7 +17760,7 @@
       </c>
       <c r="K315" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17815,7 +17815,7 @@
       </c>
       <c r="K316" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17870,7 +17870,7 @@
       </c>
       <c r="K317" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17925,7 +17925,7 @@
       </c>
       <c r="K318" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -17980,7 +17980,7 @@
       </c>
       <c r="K319" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18035,7 +18035,7 @@
       </c>
       <c r="K320" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18090,7 +18090,7 @@
       </c>
       <c r="K321" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18145,7 +18145,7 @@
       </c>
       <c r="K322" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18200,7 +18200,7 @@
       </c>
       <c r="K323" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18255,7 +18255,7 @@
       </c>
       <c r="K324" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18310,7 +18310,7 @@
       </c>
       <c r="K325" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18365,7 +18365,7 @@
       </c>
       <c r="K326" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18420,7 +18420,7 @@
       </c>
       <c r="K327" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18475,7 +18475,7 @@
       </c>
       <c r="K328" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18530,7 +18530,7 @@
       </c>
       <c r="K329" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18585,7 +18585,7 @@
       </c>
       <c r="K330" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18640,7 +18640,7 @@
       </c>
       <c r="K331" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18695,7 +18695,7 @@
       </c>
       <c r="K332" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18750,7 +18750,7 @@
       </c>
       <c r="K333" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18805,7 +18805,7 @@
       </c>
       <c r="K334" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18860,7 +18860,7 @@
       </c>
       <c r="K335" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18915,7 +18915,7 @@
       </c>
       <c r="K336" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -18970,7 +18970,7 @@
       </c>
       <c r="K337" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19025,7 +19025,7 @@
       </c>
       <c r="K338" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19080,7 +19080,7 @@
       </c>
       <c r="K339" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19135,7 +19135,7 @@
       </c>
       <c r="K340" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19190,7 +19190,7 @@
       </c>
       <c r="K341" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19245,7 +19245,7 @@
       </c>
       <c r="K342" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19300,7 +19300,7 @@
       </c>
       <c r="K343" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19355,7 +19355,7 @@
       </c>
       <c r="K344" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19410,7 +19410,7 @@
       </c>
       <c r="K345" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19465,7 +19465,7 @@
       </c>
       <c r="K346" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19520,7 +19520,7 @@
       </c>
       <c r="K347" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19575,7 +19575,7 @@
       </c>
       <c r="K348" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19630,7 +19630,7 @@
       </c>
       <c r="K349" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19685,7 +19685,7 @@
       </c>
       <c r="K350" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19740,7 +19740,7 @@
       </c>
       <c r="K351" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19795,7 +19795,7 @@
       </c>
       <c r="K352" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19850,7 +19850,7 @@
       </c>
       <c r="K353" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19905,7 +19905,7 @@
       </c>
       <c r="K354" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -19960,7 +19960,7 @@
       </c>
       <c r="K355" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20015,7 +20015,7 @@
       </c>
       <c r="K356" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20070,7 +20070,7 @@
       </c>
       <c r="K357" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20125,7 +20125,7 @@
       </c>
       <c r="K358" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20180,7 +20180,7 @@
       </c>
       <c r="K359" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20235,7 +20235,7 @@
       </c>
       <c r="K360" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20290,7 +20290,7 @@
       </c>
       <c r="K361" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20345,7 +20345,7 @@
       </c>
       <c r="K362" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20400,7 +20400,7 @@
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20455,7 +20455,7 @@
       </c>
       <c r="K364" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20510,7 +20510,7 @@
       </c>
       <c r="K365" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20565,7 +20565,7 @@
       </c>
       <c r="K366" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20620,7 +20620,7 @@
       </c>
       <c r="K367" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20675,7 +20675,7 @@
       </c>
       <c r="K368" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20730,7 +20730,7 @@
       </c>
       <c r="K369" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20785,7 +20785,7 @@
       </c>
       <c r="K370" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20840,7 +20840,7 @@
       </c>
       <c r="K371" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20895,7 +20895,7 @@
       </c>
       <c r="K372" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -20950,7 +20950,7 @@
       </c>
       <c r="K373" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21005,7 +21005,7 @@
       </c>
       <c r="K374" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21060,7 +21060,7 @@
       </c>
       <c r="K375" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21115,7 +21115,7 @@
       </c>
       <c r="K376" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21170,7 +21170,7 @@
       </c>
       <c r="K377" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21225,7 +21225,7 @@
       </c>
       <c r="K378" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21280,7 +21280,7 @@
       </c>
       <c r="K379" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21335,7 +21335,7 @@
       </c>
       <c r="K380" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21390,7 +21390,7 @@
       </c>
       <c r="K381" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21445,7 +21445,7 @@
       </c>
       <c r="K382" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21500,7 +21500,7 @@
       </c>
       <c r="K383" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21555,7 +21555,7 @@
       </c>
       <c r="K384" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21610,7 +21610,7 @@
       </c>
       <c r="K385" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21665,7 +21665,7 @@
       </c>
       <c r="K386" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21720,7 +21720,7 @@
       </c>
       <c r="K387" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21775,7 +21775,7 @@
       </c>
       <c r="K388" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21830,7 +21830,7 @@
       </c>
       <c r="K389" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21885,7 +21885,7 @@
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21940,7 +21940,7 @@
       </c>
       <c r="K391" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -21995,7 +21995,7 @@
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22050,7 +22050,7 @@
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22105,7 +22105,7 @@
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22160,7 +22160,7 @@
       </c>
       <c r="K395" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22215,7 +22215,7 @@
       </c>
       <c r="K396" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22270,7 +22270,7 @@
       </c>
       <c r="K397" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22325,7 +22325,7 @@
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22380,7 +22380,7 @@
       </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22435,7 +22435,7 @@
       </c>
       <c r="K400" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22490,7 +22490,7 @@
       </c>
       <c r="K401" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22545,7 +22545,7 @@
       </c>
       <c r="K402" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22600,7 +22600,7 @@
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22655,7 +22655,7 @@
       </c>
       <c r="K404" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22710,7 +22710,7 @@
       </c>
       <c r="K405" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22765,7 +22765,7 @@
       </c>
       <c r="K406" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22820,7 +22820,7 @@
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22875,7 +22875,7 @@
       </c>
       <c r="K408" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22930,7 +22930,7 @@
       </c>
       <c r="K409" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -22985,7 +22985,7 @@
       </c>
       <c r="K410" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23040,7 +23040,7 @@
       </c>
       <c r="K411" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23095,7 +23095,7 @@
       </c>
       <c r="K412" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23150,7 +23150,7 @@
       </c>
       <c r="K413" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23205,7 +23205,7 @@
       </c>
       <c r="K414" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23260,7 +23260,7 @@
       </c>
       <c r="K415" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23315,7 +23315,7 @@
       </c>
       <c r="K416" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23370,7 +23370,7 @@
       </c>
       <c r="K417" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23425,7 +23425,7 @@
       </c>
       <c r="K418" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23480,7 +23480,7 @@
       </c>
       <c r="K419" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23535,7 +23535,7 @@
       </c>
       <c r="K420" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23590,7 +23590,7 @@
       </c>
       <c r="K421" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23645,7 +23645,7 @@
       </c>
       <c r="K422" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23700,7 +23700,7 @@
       </c>
       <c r="K423" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23755,7 +23755,7 @@
       </c>
       <c r="K424" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23810,7 +23810,7 @@
       </c>
       <c r="K425" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23865,7 +23865,7 @@
       </c>
       <c r="K426" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23920,7 +23920,7 @@
       </c>
       <c r="K427" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -23975,7 +23975,7 @@
       </c>
       <c r="K428" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24030,7 +24030,7 @@
       </c>
       <c r="K429" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24085,7 +24085,7 @@
       </c>
       <c r="K430" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24140,7 +24140,7 @@
       </c>
       <c r="K431" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24195,7 +24195,7 @@
       </c>
       <c r="K432" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24250,7 +24250,7 @@
       </c>
       <c r="K433" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24305,7 +24305,7 @@
       </c>
       <c r="K434" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24360,7 +24360,7 @@
       </c>
       <c r="K435" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24415,7 +24415,7 @@
       </c>
       <c r="K436" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24470,7 +24470,7 @@
       </c>
       <c r="K437" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24525,7 +24525,7 @@
       </c>
       <c r="K438" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24580,7 +24580,7 @@
       </c>
       <c r="K439" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24635,7 +24635,7 @@
       </c>
       <c r="K440" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24690,7 +24690,7 @@
       </c>
       <c r="K441" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24745,7 +24745,7 @@
       </c>
       <c r="K442" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24800,7 +24800,7 @@
       </c>
       <c r="K443" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24855,7 +24855,7 @@
       </c>
       <c r="K444" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24910,7 +24910,7 @@
       </c>
       <c r="K445" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -24965,7 +24965,7 @@
       </c>
       <c r="K446" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25020,7 +25020,7 @@
       </c>
       <c r="K447" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25075,7 +25075,7 @@
       </c>
       <c r="K448" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25130,7 +25130,7 @@
       </c>
       <c r="K449" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25185,7 +25185,7 @@
       </c>
       <c r="K450" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25240,7 +25240,7 @@
       </c>
       <c r="K451" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25295,7 +25295,7 @@
       </c>
       <c r="K452" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25350,7 +25350,7 @@
       </c>
       <c r="K453" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25405,7 +25405,7 @@
       </c>
       <c r="K454" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25460,7 +25460,7 @@
       </c>
       <c r="K455" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25515,7 +25515,7 @@
       </c>
       <c r="K456" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25570,7 +25570,7 @@
       </c>
       <c r="K457" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25625,7 +25625,7 @@
       </c>
       <c r="K458" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25680,7 +25680,7 @@
       </c>
       <c r="K459" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25735,7 +25735,7 @@
       </c>
       <c r="K460" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25790,7 +25790,7 @@
       </c>
       <c r="K461" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25845,7 +25845,7 @@
       </c>
       <c r="K462" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25900,7 +25900,7 @@
       </c>
       <c r="K463" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -25955,7 +25955,7 @@
       </c>
       <c r="K464" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26010,7 +26010,7 @@
       </c>
       <c r="K465" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26065,7 +26065,7 @@
       </c>
       <c r="K466" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26120,7 +26120,7 @@
       </c>
       <c r="K467" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="K468" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26230,7 +26230,7 @@
       </c>
       <c r="K469" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26285,7 +26285,7 @@
       </c>
       <c r="K470" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26340,7 +26340,7 @@
       </c>
       <c r="K471" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26395,7 +26395,7 @@
       </c>
       <c r="K472" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26450,7 +26450,7 @@
       </c>
       <c r="K473" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26505,7 +26505,7 @@
       </c>
       <c r="K474" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26560,7 +26560,7 @@
       </c>
       <c r="K475" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26615,7 +26615,7 @@
       </c>
       <c r="K476" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26670,7 +26670,7 @@
       </c>
       <c r="K477" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26725,7 +26725,7 @@
       </c>
       <c r="K478" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26780,7 +26780,7 @@
       </c>
       <c r="K479" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26835,7 +26835,7 @@
       </c>
       <c r="K480" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26890,7 +26890,7 @@
       </c>
       <c r="K481" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -26945,7 +26945,7 @@
       </c>
       <c r="K482" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27000,7 +27000,7 @@
       </c>
       <c r="K483" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27055,7 +27055,7 @@
       </c>
       <c r="K484" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27110,7 +27110,7 @@
       </c>
       <c r="K485" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27165,7 +27165,7 @@
       </c>
       <c r="K486" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27220,7 +27220,7 @@
       </c>
       <c r="K487" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27275,7 +27275,7 @@
       </c>
       <c r="K488" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27330,7 +27330,7 @@
       </c>
       <c r="K489" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27385,7 +27385,7 @@
       </c>
       <c r="K490" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27440,7 +27440,7 @@
       </c>
       <c r="K491" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27495,7 +27495,7 @@
       </c>
       <c r="K492" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27550,7 +27550,7 @@
       </c>
       <c r="K493" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27605,7 +27605,7 @@
       </c>
       <c r="K494" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27660,7 +27660,7 @@
       </c>
       <c r="K495" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27715,7 +27715,7 @@
       </c>
       <c r="K496" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27770,7 +27770,7 @@
       </c>
       <c r="K497" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27825,7 +27825,7 @@
       </c>
       <c r="K498" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27880,7 +27880,7 @@
       </c>
       <c r="K499" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27935,7 +27935,7 @@
       </c>
       <c r="K500" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -27990,7 +27990,7 @@
       </c>
       <c r="K501" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -28162,7 +28162,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Adapted from Statistics Canada, &lt;table name/number&gt;, &lt;reference date&gt;. This does not constitute an endorsement by Statistics Canada of this product.</t>
+          <t>Adapted from Statistics Canada, 2026-08. This does not constitute an endorsement by Statistics Canada of this product.</t>
         </is>
       </c>
     </row>
@@ -28198,7 +28198,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>

</xml_diff>